<commit_message>
Complete manual test execution
</commit_message>
<xml_diff>
--- a/Manual-Testing/Test Cases.xlsx
+++ b/Manual-Testing/Test Cases.xlsx
@@ -8,17 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my projects\QA Projects\SauceDemo-QA\Manual-Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E04261F-B3D4-4A9E-8305-10A165008EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9BF7CC1-1959-4D09-B4E4-C6443359922B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -28,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="294">
   <si>
     <t>Preconditions</t>
   </si>
@@ -633,9 +642,6 @@
     <t>User is on the SauceDemo login page</t>
   </si>
   <si>
-    <t>Username: standard_user Password: valid password</t>
-  </si>
-  <si>
     <t>User is redirected to the Products page</t>
   </si>
   <si>
@@ -645,9 +651,6 @@
     <t>User is on the login page</t>
   </si>
   <si>
-    <t>Username: invalid_user Password: valid password</t>
-  </si>
-  <si>
     <t>Login attempt is rejected</t>
   </si>
   <si>
@@ -657,15 +660,9 @@
     <t>Verify login with invalid password</t>
   </si>
   <si>
-    <t>Username: standard_user Password: invalid password</t>
-  </si>
-  <si>
     <t>Verify login with empty username</t>
   </si>
   <si>
-    <t>Username: blank Password: valid password</t>
-  </si>
-  <si>
     <t>Username validation message is displayed</t>
   </si>
   <si>
@@ -679,9 +676,6 @@
   </si>
   <si>
     <t>Verify locked-out user cannot log in</t>
-  </si>
-  <si>
-    <t>Username: locked_out_user Password: valid password</t>
   </si>
   <si>
     <t>User remains logged out</t>
@@ -906,6 +900,97 @@
     <t>1. Enter username 
 2. Leave password empty 
 3. Click Login</t>
+  </si>
+  <si>
+    <t>Tested By</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Username: standard_user Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Username: standard_user Password: invalid_password</t>
+  </si>
+  <si>
+    <t>Username: blank 
+Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Username: locked_out_user Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Username:  invalid_user
+Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Dasun Anjana</t>
+  </si>
+  <si>
+    <t>Successfully Login</t>
+  </si>
+  <si>
+    <t>Executed</t>
+  </si>
+  <si>
+    <t>User successfully logged
+ in and Products page was displayed</t>
+  </si>
+  <si>
+    <t>Faild Login</t>
+  </si>
+  <si>
+    <t>Available products displayed</t>
+  </si>
+  <si>
+    <t>Product details displayed correctly</t>
+  </si>
+  <si>
+    <t>Both product added to cart and cart count displayed correctly</t>
+  </si>
+  <si>
+    <t>Selected product added 
+to cart</t>
+  </si>
+  <si>
+    <t>Products are sorted 
+correctly</t>
+  </si>
+  <si>
+    <t>Cart count displayed 
+correctly</t>
+  </si>
+  <si>
+    <t>Product name, price and 
+details are displayed</t>
+  </si>
+  <si>
+    <t>Cart displayed correct product quantity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product is removed </t>
+  </si>
+  <si>
+    <t>Multiple products are removed</t>
+  </si>
+  <si>
+    <t>Products are displayed</t>
+  </si>
+  <si>
+    <t>Navigated to Checkout: Your Information page</t>
+  </si>
+  <si>
+    <t>Failed Checkout</t>
+  </si>
+  <si>
+    <t>Checkout details shows</t>
+  </si>
+  <si>
+    <t>Calculations are correct</t>
+  </si>
+  <si>
+    <t>Order placed successfully</t>
   </si>
 </sst>
 </file>
@@ -951,12 +1036,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -969,12 +1048,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1002,11 +1087,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1020,23 +1114,47 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1318,7 +1436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.5546875" customWidth="1"/>
@@ -1329,15 +1447,18 @@
     <col min="6" max="6" width="31.109375" customWidth="1"/>
     <col min="7" max="7" width="26.21875" customWidth="1"/>
     <col min="8" max="8" width="21.109375" customWidth="1"/>
-    <col min="9" max="9" width="22.109375" customWidth="1"/>
-    <col min="10" max="10" width="22.21875" customWidth="1"/>
+    <col min="9" max="9" width="24.21875" customWidth="1"/>
+    <col min="10" max="10" width="24.5546875" style="14" customWidth="1"/>
     <col min="11" max="11" width="20.77734375" customWidth="1"/>
     <col min="12" max="12" width="19.77734375" customWidth="1"/>
     <col min="13" max="13" width="24.6640625" customWidth="1"/>
-    <col min="14" max="14" width="21.88671875" customWidth="1"/>
+    <col min="14" max="14" width="21.88671875" style="14" customWidth="1"/>
+    <col min="15" max="15" width="19.77734375" style="14" customWidth="1"/>
+    <col min="16" max="16" width="22.21875" style="14" customWidth="1"/>
+    <col min="17" max="17" width="21.6640625" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>188</v>
       </c>
@@ -1365,7 +1486,7 @@
       <c r="I1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="13" t="s">
         <v>194</v>
       </c>
       <c r="K1" s="2" t="s">
@@ -1377,11 +1498,20 @@
       <c r="M1" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="13" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O1" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="P1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q1" s="15" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1398,22 +1528,24 @@
         <v>200</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="J2" s="1"/>
-      <c r="K2" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L2" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M2" s="1" t="s">
@@ -1422,8 +1554,17 @@
       <c r="N2" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O2" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="P2" s="11">
+        <v>46277</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1434,28 +1575,30 @@
         <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="J3" s="1"/>
-      <c r="K3" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L3" s="4" t="s">
+      <c r="J3" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M3" s="1" t="s">
@@ -1464,8 +1607,17 @@
       <c r="N3" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O3" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P3" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q3" s="8" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -1476,28 +1628,30 @@
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>206</v>
-      </c>
       <c r="I4" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="J4" s="1"/>
-      <c r="K4" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L4" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M4" s="1" t="s">
@@ -1506,8 +1660,17 @@
       <c r="N4" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O4" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P4" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q4" s="8" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -1518,28 +1681,30 @@
         <v>12</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>206</v>
-      </c>
       <c r="I5" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="J5" s="1"/>
-      <c r="K5" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L5" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M5" s="1" t="s">
@@ -1548,8 +1713,17 @@
       <c r="N5" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O5" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P5" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q5" s="8" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1560,28 +1734,30 @@
         <v>14</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>206</v>
-      </c>
       <c r="I6" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="J6" s="1"/>
-      <c r="K6" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L6" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M6" s="1" t="s">
@@ -1590,8 +1766,17 @@
       <c r="N6" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O6" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P6" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q6" s="8" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -1602,28 +1787,30 @@
         <v>16</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>217</v>
+        <v>271</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="J7" s="1"/>
-      <c r="K7" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L7" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M7" s="1" t="s">
@@ -1632,8 +1819,17 @@
       <c r="N7" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O7" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P7" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q7" s="8" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -1644,28 +1840,30 @@
         <v>18</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="J8" s="1"/>
-      <c r="K8" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L8" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M8" s="1" t="s">
@@ -1674,8 +1872,17 @@
       <c r="N8" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O8" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P8" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q8" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
@@ -1692,22 +1899,24 @@
         <v>23</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>97</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="J9" s="1"/>
-      <c r="K9" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L9" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L9" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M9" s="1" t="s">
@@ -1716,8 +1925,17 @@
       <c r="N9" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O9" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P9" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q9" s="8" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
@@ -1728,16 +1946,16 @@
         <v>26</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>91</v>
@@ -1745,11 +1963,13 @@
       <c r="I10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J10" s="1"/>
-      <c r="K10" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L10" s="5" t="s">
+      <c r="J10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L10" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M10" s="1" t="s">
@@ -1758,8 +1978,17 @@
       <c r="N10" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O10" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P10" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q10" s="12" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>28</v>
       </c>
@@ -1776,7 +2005,7 @@
         <v>23</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>90</v>
@@ -1787,11 +2016,13 @@
       <c r="I11" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="J11" s="1"/>
-      <c r="K11" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L11" s="5" t="s">
+      <c r="J11" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L11" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M11" s="1" t="s">
@@ -1800,8 +2031,17 @@
       <c r="N11" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O11" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P11" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q11" s="12" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
@@ -1818,7 +2058,7 @@
         <v>23</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>97</v>
@@ -1829,11 +2069,13 @@
       <c r="I12" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="J12" s="1"/>
-      <c r="K12" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L12" s="4" t="s">
+      <c r="J12" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M12" s="1" t="s">
@@ -1842,8 +2084,17 @@
       <c r="N12" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O12" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P12" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q12" s="12" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>32</v>
       </c>
@@ -1860,7 +2111,7 @@
         <v>23</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>102</v>
@@ -1871,11 +2122,13 @@
       <c r="I13" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="1"/>
-      <c r="K13" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L13" s="4" t="s">
+      <c r="J13" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L13" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M13" s="1" t="s">
@@ -1884,8 +2137,17 @@
       <c r="N13" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O13" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P13" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q13" s="12" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>34</v>
       </c>
@@ -1902,7 +2164,7 @@
         <v>106</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>36</v>
@@ -1913,11 +2175,13 @@
       <c r="I14" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="J14" s="1"/>
-      <c r="K14" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L14" s="5" t="s">
+      <c r="J14" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L14" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M14" s="1" t="s">
@@ -1926,8 +2190,17 @@
       <c r="N14" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O14" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P14" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q14" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>37</v>
       </c>
@@ -1944,7 +2217,7 @@
         <v>111</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>39</v>
@@ -1955,11 +2228,13 @@
       <c r="I15" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="J15" s="1"/>
-      <c r="K15" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L15" s="4" t="s">
+      <c r="J15" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L15" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M15" s="1" t="s">
@@ -1968,50 +2243,70 @@
       <c r="N15" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
+      <c r="O15" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P15" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q15" s="12" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="I16" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="D16" s="10" t="s">
-        <v>265</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="J16" s="7"/>
-      <c r="K16" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="L16" s="9" t="s">
+      <c r="J16" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L16" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M16" s="7" t="s">
+      <c r="M16" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="N16" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N16" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="O16" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P16" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q16" s="14" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>42</v>
       </c>
@@ -2028,7 +2323,7 @@
         <v>115</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>39</v>
@@ -2039,11 +2334,13 @@
       <c r="I17" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="J17" s="1"/>
-      <c r="K17" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L17" s="4" t="s">
+      <c r="J17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L17" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M17" s="1" t="s">
@@ -2052,8 +2349,17 @@
       <c r="N17" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O17" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P17" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q17" s="14" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>44</v>
       </c>
@@ -2070,7 +2376,7 @@
         <v>119</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>62</v>
@@ -2081,11 +2387,13 @@
       <c r="I18" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="J18" s="1"/>
-      <c r="K18" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L18" s="5" t="s">
+      <c r="J18" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L18" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M18" s="1" t="s">
@@ -2094,10 +2402,19 @@
       <c r="N18" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O18" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P18" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q18" s="14" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>109</v>
@@ -2123,11 +2440,13 @@
       <c r="I19" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="J19" s="1"/>
-      <c r="K19" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L19" s="5" t="s">
+      <c r="J19" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L19" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M19" s="1" t="s">
@@ -2136,8 +2455,17 @@
       <c r="N19" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O19" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P19" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q19" s="14" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>48</v>
       </c>
@@ -2154,7 +2482,7 @@
         <v>115</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>39</v>
@@ -2165,11 +2493,13 @@
       <c r="I20" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="J20" s="1"/>
-      <c r="K20" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L20" s="4" t="s">
+      <c r="J20" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M20" s="1" t="s">
@@ -2178,8 +2508,17 @@
       <c r="N20" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O20" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P20" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q20" s="14" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>50</v>
       </c>
@@ -2196,10 +2535,10 @@
         <v>131</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>132</v>
@@ -2207,11 +2546,13 @@
       <c r="I21" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="J21" s="1"/>
-      <c r="K21" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L21" s="4" t="s">
+      <c r="J21" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L21" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M21" s="1" t="s">
@@ -2220,8 +2561,17 @@
       <c r="N21" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O21" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P21" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q21" s="14" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>52</v>
       </c>
@@ -2238,10 +2588,10 @@
         <v>131</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>132</v>
@@ -2249,11 +2599,13 @@
       <c r="I22" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="J22" s="1"/>
-      <c r="K22" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L22" s="4" t="s">
+      <c r="J22" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L22" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M22" s="1" t="s">
@@ -2262,8 +2614,17 @@
       <c r="N22" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O22" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P22" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q22" s="14" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>54</v>
       </c>
@@ -2280,10 +2641,10 @@
         <v>131</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="H23" s="1" t="s">
         <v>132</v>
@@ -2291,11 +2652,13 @@
       <c r="I23" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="J23" s="1"/>
-      <c r="K23" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L23" s="4" t="s">
+      <c r="J23" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L23" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M23" s="1" t="s">
@@ -2304,8 +2667,17 @@
       <c r="N23" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O23" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P23" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q23" s="14" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>56</v>
       </c>
@@ -2322,10 +2694,10 @@
         <v>139</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>140</v>
@@ -2333,11 +2705,13 @@
       <c r="I24" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="J24" s="1"/>
-      <c r="K24" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L24" s="4" t="s">
+      <c r="J24" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L24" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M24" s="1" t="s">
@@ -2346,8 +2720,17 @@
       <c r="N24" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O24" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P24" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q24" s="14" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>58</v>
       </c>
@@ -2364,7 +2747,7 @@
         <v>143</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>144</v>
@@ -2375,11 +2758,13 @@
       <c r="I25" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="J25" s="1"/>
-      <c r="K25" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L25" s="4" t="s">
+      <c r="J25" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M25" s="1" t="s">
@@ -2388,8 +2773,14 @@
       <c r="N25" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O25" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P25" s="9">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>60</v>
       </c>
@@ -2406,7 +2797,7 @@
         <v>148</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>149</v>
@@ -2417,11 +2808,13 @@
       <c r="I26" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="J26" s="1"/>
-      <c r="K26" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L26" s="4" t="s">
+      <c r="J26" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L26" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M26" s="1" t="s">
@@ -2430,8 +2823,17 @@
       <c r="N26" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O26" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P26" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q26" s="14" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>64</v>
       </c>
@@ -2448,7 +2850,7 @@
         <v>148</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>151</v>
@@ -2459,11 +2861,13 @@
       <c r="I27" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="J27" s="1"/>
-      <c r="K27" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L27" s="4" t="s">
+      <c r="J27" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L27" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M27" s="1" t="s">
@@ -2472,8 +2876,17 @@
       <c r="N27" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O27" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P27" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q27" s="14" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>67</v>
       </c>
@@ -2490,7 +2903,7 @@
         <v>148</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>154</v>
@@ -2501,11 +2914,13 @@
       <c r="I28" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="J28" s="1"/>
-      <c r="K28" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L28" s="4" t="s">
+      <c r="J28" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L28" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M28" s="1" t="s">
@@ -2514,8 +2929,17 @@
       <c r="N28" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O28" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P28" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q28" s="14" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>69</v>
       </c>
@@ -2532,7 +2956,7 @@
         <v>157</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>158</v>
@@ -2543,11 +2967,13 @@
       <c r="I29" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J29" s="1"/>
-      <c r="K29" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L29" s="6" t="s">
+      <c r="J29" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L29" s="16" t="s">
         <v>71</v>
       </c>
       <c r="M29" s="1" t="s">
@@ -2556,8 +2982,17 @@
       <c r="N29" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O29" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P29" s="9">
+        <v>46277</v>
+      </c>
+      <c r="Q29" s="14" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>72</v>
       </c>
@@ -2585,11 +3020,13 @@
       <c r="I30" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="J30" s="1"/>
-      <c r="K30" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L30" s="4" t="s">
+      <c r="J30" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L30" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M30" s="1" t="s">
@@ -2598,8 +3035,14 @@
       <c r="N30" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O30" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P30" s="9">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>75</v>
       </c>
@@ -2627,11 +3070,13 @@
       <c r="I31" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="J31" s="1"/>
-      <c r="K31" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L31" s="5" t="s">
+      <c r="J31" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="K31" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L31" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M31" s="1" t="s">
@@ -2640,8 +3085,14 @@
       <c r="N31" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O31" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P31" s="9">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>77</v>
       </c>
@@ -2658,7 +3109,7 @@
         <v>19</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>47</v>
@@ -2669,11 +3120,13 @@
       <c r="I32" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J32" s="1"/>
-      <c r="K32" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L32" s="4" t="s">
+      <c r="J32" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L32" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M32" s="1" t="s">
@@ -2682,8 +3135,14 @@
       <c r="N32" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="33" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O32" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P32" s="9">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>79</v>
       </c>
@@ -2700,7 +3159,7 @@
         <v>19</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="G33" s="1" t="s">
         <v>47</v>
@@ -2711,11 +3170,13 @@
       <c r="I33" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="J33" s="1"/>
-      <c r="K33" s="3" t="s">
+      <c r="J33" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="K33" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="L33" s="5" t="s">
+      <c r="L33" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M33" s="1" t="s">
@@ -2724,8 +3185,14 @@
       <c r="N33" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O33" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P33" s="9">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>82</v>
       </c>
@@ -2742,7 +3209,7 @@
         <v>23</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>47</v>
@@ -2753,11 +3220,13 @@
       <c r="I34" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="J34" s="1"/>
-      <c r="K34" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L34" s="5" t="s">
+      <c r="J34" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="L34" s="17" t="s">
         <v>24</v>
       </c>
       <c r="M34" s="1" t="s">
@@ -2766,8 +3235,14 @@
       <c r="N34" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O34" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P34" s="9">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>84</v>
       </c>
@@ -2784,7 +3259,7 @@
         <v>182</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>183</v>
@@ -2795,11 +3270,13 @@
       <c r="I35" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="J35" s="1"/>
-      <c r="K35" s="3" t="s">
+      <c r="J35" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="K35" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="L35" s="4" t="s">
+      <c r="L35" s="3" t="s">
         <v>6</v>
       </c>
       <c r="M35" s="1" t="s">
@@ -2808,8 +3285,14 @@
       <c r="N35" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O35" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P35" s="9">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>86</v>
       </c>
@@ -2826,7 +3309,7 @@
         <v>182</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>186</v>
@@ -2837,11 +3320,13 @@
       <c r="I36" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="J36" s="1"/>
-      <c r="K36" s="3" t="s">
+      <c r="J36" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="K36" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="L36" s="6" t="s">
+      <c r="L36" s="16" t="s">
         <v>71</v>
       </c>
       <c r="M36" s="1" t="s">
@@ -2849,6 +3334,12 @@
       </c>
       <c r="N36" s="1" t="s">
         <v>95</v>
+      </c>
+      <c r="O36" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="P36" s="9">
+        <v>46277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>